<commit_message>
Add dealerlist active status source
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -4942,7 +4942,7 @@
       </c>
       <c r="AF43" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="AF44" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5254,7 +5254,7 @@
       </c>
       <c r="AF46" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5358,7 @@
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -10754,7 +10754,7 @@
       </c>
       <c r="AF99" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -10858,7 +10858,7 @@
       </c>
       <c r="AF100" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -10962,7 +10962,7 @@
       </c>
       <c r="AF101" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -13978,7 +13978,7 @@
       </c>
       <c r="AF130" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -14082,7 +14082,7 @@
       </c>
       <c r="AF131" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -14186,7 +14186,7 @@
       </c>
       <c r="AF132" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -21154,7 +21154,7 @@
       </c>
       <c r="AF199" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
@@ -21258,7 +21258,7 @@
       </c>
       <c r="AF200" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
@@ -21362,7 +21362,7 @@
       </c>
       <c r="AF201" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
@@ -21466,7 +21466,7 @@
       </c>
       <c r="AF202" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
@@ -21570,7 +21570,7 @@
       </c>
       <c r="AF203" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="AF204" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
@@ -22714,7 +22714,7 @@
       </c>
       <c r="AF214" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
@@ -22818,7 +22818,7 @@
       </c>
       <c r="AF215" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
@@ -22922,7 +22922,7 @@
       </c>
       <c r="AF216" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -23026,7 +23026,7 @@
       </c>
       <c r="AF217" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -23130,7 +23130,7 @@
       </c>
       <c r="AF218" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Merge Rothwell into Redcliffe
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF224"/>
+  <dimension ref="A1:AF220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17949,7 +17949,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E169" t="n">
         <v>0</v>
@@ -17997,7 +17997,7 @@
         <v>0</v>
       </c>
       <c r="T169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U169" t="n">
         <v>0</v>
@@ -18053,7 +18053,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E170" t="n">
         <v>0</v>
@@ -18157,7 +18157,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E171" t="n">
         <v>0</v>
@@ -18184,7 +18184,7 @@
         <v>0</v>
       </c>
       <c r="M171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N171" t="n">
         <v>0</v>
@@ -18413,7 +18413,7 @@
         <v>0</v>
       </c>
       <c r="T173" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U173" t="n">
         <v>0</v>
@@ -19184,11 +19184,11 @@
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>140221</v>
+        <v>136301</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Rothwell</t>
+          <t>Shepparton</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -19197,7 +19197,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E181" t="n">
         <v>0</v>
@@ -19206,7 +19206,7 @@
         <v>0</v>
       </c>
       <c r="G181" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H181" t="n">
         <v>0</v>
@@ -19245,7 +19245,7 @@
         <v>0</v>
       </c>
       <c r="T181" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U181" t="n">
         <v>0</v>
@@ -19288,11 +19288,11 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>140221</v>
+        <v>136301</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Rothwell</t>
+          <t>Shepparton</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -19301,10 +19301,10 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E182" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F182" t="n">
         <v>0</v>
@@ -19367,7 +19367,7 @@
         <v>0</v>
       </c>
       <c r="Z182" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA182" t="n">
         <v>0</v>
@@ -19392,11 +19392,11 @@
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>140221</v>
+        <v>136301</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Rothwell</t>
+          <t>Shepparton</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -19405,7 +19405,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E183" t="n">
         <v>0</v>
@@ -19432,7 +19432,7 @@
         <v>0</v>
       </c>
       <c r="M183" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N183" t="n">
         <v>0</v>
@@ -19468,7 +19468,7 @@
         <v>0</v>
       </c>
       <c r="Y183" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z183" t="n">
         <v>0</v>
@@ -19496,16 +19496,16 @@
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>140221</v>
+        <v>136301</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Rothwell</t>
+          <t>Shepparton</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -19557,7 +19557,7 @@
         <v>0</v>
       </c>
       <c r="T184" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U184" t="n">
         <v>0</v>
@@ -19575,7 +19575,7 @@
         <v>0</v>
       </c>
       <c r="Z184" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AA184" t="n">
         <v>0</v>
@@ -19609,7 +19609,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>May</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -19622,7 +19622,7 @@
         <v>0</v>
       </c>
       <c r="G185" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H185" t="n">
         <v>0</v>
@@ -19676,10 +19676,10 @@
         <v>0</v>
       </c>
       <c r="Y185" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z185" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA185" t="n">
         <v>0</v>
@@ -19713,14 +19713,14 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E186" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F186" t="n">
         <v>0</v>
@@ -19783,7 +19783,7 @@
         <v>0</v>
       </c>
       <c r="Z186" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AA186" t="n">
         <v>0</v>
@@ -19808,20 +19808,20 @@
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>136301</v>
+        <v>141271</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Shepparton</t>
+          <t>Springwood</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E187" t="n">
         <v>0</v>
@@ -19887,7 +19887,7 @@
         <v>1</v>
       </c>
       <c r="Z187" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA187" t="n">
         <v>0</v>
@@ -19912,20 +19912,20 @@
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>136301</v>
+        <v>141271</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Shepparton</t>
+          <t>Springwood</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E188" t="n">
         <v>0</v>
@@ -19973,7 +19973,7 @@
         <v>0</v>
       </c>
       <c r="T188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U188" t="n">
         <v>0</v>
@@ -19988,16 +19988,16 @@
         <v>0</v>
       </c>
       <c r="Y188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z188" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AA188" t="n">
         <v>0</v>
       </c>
       <c r="AB188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC188" t="n">
         <v>0</v>
@@ -20016,16 +20016,16 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>136301</v>
+        <v>141271</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Shepparton</t>
+          <t>Springwood</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -20095,7 +20095,7 @@
         <v>1</v>
       </c>
       <c r="Z189" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA189" t="n">
         <v>0</v>
@@ -20120,16 +20120,16 @@
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>136301</v>
+        <v>141271</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Shepparton</t>
+          <t>Springwood</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -20199,7 +20199,7 @@
         <v>0</v>
       </c>
       <c r="Z190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA190" t="n">
         <v>0</v>
@@ -20233,11 +20233,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>May</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E191" t="n">
         <v>0</v>
@@ -20300,7 +20300,7 @@
         <v>0</v>
       </c>
       <c r="Y191" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Z191" t="n">
         <v>1</v>
@@ -20328,20 +20328,20 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>141271</v>
+        <v>123401</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Springwood</t>
+          <t>Tamworth</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E192" t="n">
         <v>0</v>
@@ -20389,7 +20389,7 @@
         <v>0</v>
       </c>
       <c r="T192" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U192" t="n">
         <v>0</v>
@@ -20404,16 +20404,16 @@
         <v>0</v>
       </c>
       <c r="Y192" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z192" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA192" t="n">
         <v>0</v>
       </c>
       <c r="AB192" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC192" t="n">
         <v>0</v>
@@ -20432,16 +20432,16 @@
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>141271</v>
+        <v>123401</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Springwood</t>
+          <t>Tamworth</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -20490,7 +20490,7 @@
         <v>0</v>
       </c>
       <c r="S193" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T193" t="n">
         <v>0</v>
@@ -20508,10 +20508,10 @@
         <v>0</v>
       </c>
       <c r="Y193" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z193" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA193" t="n">
         <v>0</v>
@@ -20536,29 +20536,29 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>141271</v>
+        <v>123401</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Springwood</t>
+          <t>Tamworth</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>May</t>
         </is>
       </c>
       <c r="D194" t="n">
         <v>0</v>
       </c>
       <c r="E194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F194" t="n">
         <v>0</v>
       </c>
       <c r="G194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H194" t="n">
         <v>0</v>
@@ -20615,7 +20615,7 @@
         <v>0</v>
       </c>
       <c r="Z194" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA194" t="n">
         <v>0</v>
@@ -20640,20 +20640,20 @@
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>141271</v>
+        <v>143501</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Springwood</t>
+          <t>Toowoomba</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E195" t="n">
         <v>0</v>
@@ -20716,13 +20716,13 @@
         <v>0</v>
       </c>
       <c r="Y195" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA195" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB195" t="n">
         <v>0</v>
@@ -20738,17 +20738,17 @@
       </c>
       <c r="AF195" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>123401</v>
+        <v>143501</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Tamworth</t>
+          <t>Toowoomba</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -20757,7 +20757,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E196" t="n">
         <v>0</v>
@@ -20790,7 +20790,7 @@
         <v>0</v>
       </c>
       <c r="O196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P196" t="n">
         <v>0</v>
@@ -20842,22 +20842,22 @@
       </c>
       <c r="AF196" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>123401</v>
+        <v>148141</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Tamworth</t>
+          <t>Townsville</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -20906,10 +20906,10 @@
         <v>0</v>
       </c>
       <c r="S197" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T197" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U197" t="n">
         <v>0</v>
@@ -20927,10 +20927,10 @@
         <v>0</v>
       </c>
       <c r="Z197" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA197" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB197" t="n">
         <v>0</v>
@@ -20946,35 +20946,35 @@
       </c>
       <c r="AF197" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>123401</v>
+        <v>148141</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Tamworth</t>
+          <t>Townsville</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E198" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F198" t="n">
         <v>0</v>
       </c>
       <c r="G198" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H198" t="n">
         <v>0</v>
@@ -21037,7 +21037,7 @@
         <v>0</v>
       </c>
       <c r="AB198" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC198" t="n">
         <v>0</v>
@@ -21050,22 +21050,22 @@
       </c>
       <c r="AF198" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>143501</v>
+        <v>148141</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Toowoomba</t>
+          <t>Townsville</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -21132,16 +21132,16 @@
         <v>0</v>
       </c>
       <c r="Y199" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z199" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AA199" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB199" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC199" t="n">
         <v>0</v>
@@ -21160,16 +21160,16 @@
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>143501</v>
+        <v>148141</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Toowoomba</t>
+          <t>Townsville</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -21206,7 +21206,7 @@
         <v>0</v>
       </c>
       <c r="O200" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P200" t="n">
         <v>0</v>
@@ -21239,7 +21239,7 @@
         <v>0</v>
       </c>
       <c r="Z200" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AA200" t="n">
         <v>0</v>
@@ -21264,11 +21264,11 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>148141</v>
+        <v>122591</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Townsville</t>
+          <t>Tuggerah</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -21277,7 +21277,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E201" t="n">
         <v>0</v>
@@ -21286,7 +21286,7 @@
         <v>0</v>
       </c>
       <c r="G201" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H201" t="n">
         <v>0</v>
@@ -21328,7 +21328,7 @@
         <v>1</v>
       </c>
       <c r="U201" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V201" t="n">
         <v>0</v>
@@ -21346,7 +21346,7 @@
         <v>1</v>
       </c>
       <c r="AA201" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB201" t="n">
         <v>0</v>
@@ -21362,17 +21362,17 @@
       </c>
       <c r="AF201" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>148141</v>
+        <v>122591</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Townsville</t>
+          <t>Tuggerah</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -21381,7 +21381,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E202" t="n">
         <v>0</v>
@@ -21414,10 +21414,10 @@
         <v>0</v>
       </c>
       <c r="O202" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P202" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q202" t="n">
         <v>0</v>
@@ -21447,13 +21447,13 @@
         <v>0</v>
       </c>
       <c r="Z202" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA202" t="n">
         <v>0</v>
       </c>
       <c r="AB202" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC202" t="n">
         <v>0</v>
@@ -21466,17 +21466,17 @@
       </c>
       <c r="AF202" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>148141</v>
+        <v>122591</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Townsville</t>
+          <t>Tuggerah</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -21533,13 +21533,13 @@
         <v>0</v>
       </c>
       <c r="T203" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U203" t="n">
         <v>0</v>
       </c>
       <c r="V203" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W203" t="n">
         <v>0</v>
@@ -21548,10 +21548,10 @@
         <v>0</v>
       </c>
       <c r="Y203" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z203" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA203" t="n">
         <v>0</v>
@@ -21570,17 +21570,17 @@
       </c>
       <c r="AF203" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>148141</v>
+        <v>122591</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Townsville</t>
+          <t>Tuggerah</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -21589,7 +21589,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E204" t="n">
         <v>0</v>
@@ -21622,7 +21622,7 @@
         <v>0</v>
       </c>
       <c r="O204" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P204" t="n">
         <v>0</v>
@@ -21655,7 +21655,7 @@
         <v>0</v>
       </c>
       <c r="Z204" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA204" t="n">
         <v>0</v>
@@ -21674,7 +21674,7 @@
       </c>
       <c r="AF204" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -21689,83 +21689,83 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>May</t>
         </is>
       </c>
       <c r="D205" t="n">
+        <v>0</v>
+      </c>
+      <c r="E205" t="n">
+        <v>0</v>
+      </c>
+      <c r="F205" t="n">
+        <v>0</v>
+      </c>
+      <c r="G205" t="n">
+        <v>1</v>
+      </c>
+      <c r="H205" t="n">
+        <v>0</v>
+      </c>
+      <c r="I205" t="n">
+        <v>0</v>
+      </c>
+      <c r="J205" t="n">
+        <v>0</v>
+      </c>
+      <c r="K205" t="n">
+        <v>0</v>
+      </c>
+      <c r="L205" t="n">
+        <v>0</v>
+      </c>
+      <c r="M205" t="n">
+        <v>0</v>
+      </c>
+      <c r="N205" t="n">
+        <v>0</v>
+      </c>
+      <c r="O205" t="n">
+        <v>0</v>
+      </c>
+      <c r="P205" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q205" t="n">
+        <v>0</v>
+      </c>
+      <c r="R205" t="n">
+        <v>0</v>
+      </c>
+      <c r="S205" t="n">
+        <v>0</v>
+      </c>
+      <c r="T205" t="n">
+        <v>0</v>
+      </c>
+      <c r="U205" t="n">
+        <v>0</v>
+      </c>
+      <c r="V205" t="n">
+        <v>0</v>
+      </c>
+      <c r="W205" t="n">
+        <v>0</v>
+      </c>
+      <c r="X205" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y205" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z205" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA205" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB205" t="n">
         <v>2</v>
-      </c>
-      <c r="E205" t="n">
-        <v>0</v>
-      </c>
-      <c r="F205" t="n">
-        <v>0</v>
-      </c>
-      <c r="G205" t="n">
-        <v>1</v>
-      </c>
-      <c r="H205" t="n">
-        <v>0</v>
-      </c>
-      <c r="I205" t="n">
-        <v>0</v>
-      </c>
-      <c r="J205" t="n">
-        <v>0</v>
-      </c>
-      <c r="K205" t="n">
-        <v>0</v>
-      </c>
-      <c r="L205" t="n">
-        <v>0</v>
-      </c>
-      <c r="M205" t="n">
-        <v>0</v>
-      </c>
-      <c r="N205" t="n">
-        <v>0</v>
-      </c>
-      <c r="O205" t="n">
-        <v>0</v>
-      </c>
-      <c r="P205" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q205" t="n">
-        <v>0</v>
-      </c>
-      <c r="R205" t="n">
-        <v>0</v>
-      </c>
-      <c r="S205" t="n">
-        <v>0</v>
-      </c>
-      <c r="T205" t="n">
-        <v>1</v>
-      </c>
-      <c r="U205" t="n">
-        <v>1</v>
-      </c>
-      <c r="V205" t="n">
-        <v>0</v>
-      </c>
-      <c r="W205" t="n">
-        <v>0</v>
-      </c>
-      <c r="X205" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y205" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z205" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB205" t="n">
-        <v>0</v>
       </c>
       <c r="AC205" t="n">
         <v>0</v>
@@ -21793,7 +21793,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -21830,10 +21830,10 @@
         <v>0</v>
       </c>
       <c r="O206" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P206" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q206" t="n">
         <v>0</v>
@@ -21869,7 +21869,7 @@
         <v>0</v>
       </c>
       <c r="AB206" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC206" t="n">
         <v>0</v>
@@ -21888,16 +21888,16 @@
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>122591</v>
+        <v>124861</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Tuggerah</t>
+          <t>Tweed Heads</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -21949,13 +21949,13 @@
         <v>0</v>
       </c>
       <c r="T207" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U207" t="n">
         <v>0</v>
       </c>
       <c r="V207" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W207" t="n">
         <v>0</v>
@@ -21964,16 +21964,16 @@
         <v>0</v>
       </c>
       <c r="Y207" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z207" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA207" t="n">
         <v>0</v>
       </c>
       <c r="AB207" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC207" t="n">
         <v>0</v>
@@ -21992,20 +21992,20 @@
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>122591</v>
+        <v>124861</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Tuggerah</t>
+          <t>Tweed Heads</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E208" t="n">
         <v>0</v>
@@ -22038,7 +22038,7 @@
         <v>0</v>
       </c>
       <c r="O208" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P208" t="n">
         <v>0</v>
@@ -22056,7 +22056,7 @@
         <v>0</v>
       </c>
       <c r="U208" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V208" t="n">
         <v>0</v>
@@ -22077,7 +22077,7 @@
         <v>0</v>
       </c>
       <c r="AB208" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC208" t="n">
         <v>0</v>
@@ -22096,16 +22096,16 @@
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>122591</v>
+        <v>124861</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Tuggerah</t>
+          <t>Tweed Heads</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -22118,7 +22118,7 @@
         <v>0</v>
       </c>
       <c r="G209" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H209" t="n">
         <v>0</v>
@@ -22172,16 +22172,16 @@
         <v>0</v>
       </c>
       <c r="Y209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z209" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA209" t="n">
         <v>0</v>
       </c>
       <c r="AB209" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AC209" t="n">
         <v>0</v>
@@ -22200,16 +22200,16 @@
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>122591</v>
+        <v>126501</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Tuggerah</t>
+          <t>Wagga Wagga</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -22279,7 +22279,7 @@
         <v>0</v>
       </c>
       <c r="Z210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA210" t="n">
         <v>0</v>
@@ -22298,29 +22298,29 @@
       </c>
       <c r="AF210" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>124861</v>
+        <v>126501</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Tweed Heads</t>
+          <t>Wagga Wagga</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D211" t="n">
         <v>0</v>
       </c>
       <c r="E211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F211" t="n">
         <v>0</v>
@@ -22383,7 +22383,7 @@
         <v>0</v>
       </c>
       <c r="Z211" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA211" t="n">
         <v>0</v>
@@ -22402,26 +22402,26 @@
       </c>
       <c r="AF211" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>124861</v>
+        <v>132801</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Tweed Heads</t>
+          <t>Warrnambool</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E212" t="n">
         <v>0</v>
@@ -22472,7 +22472,7 @@
         <v>0</v>
       </c>
       <c r="U212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V212" t="n">
         <v>0</v>
@@ -22493,7 +22493,7 @@
         <v>0</v>
       </c>
       <c r="AB212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC212" t="n">
         <v>0</v>
@@ -22512,20 +22512,20 @@
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>124861</v>
+        <v>132801</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Tweed Heads</t>
+          <t>Warrnambool</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E213" t="n">
         <v>0</v>
@@ -22588,10 +22588,10 @@
         <v>0</v>
       </c>
       <c r="Y213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA213" t="n">
         <v>0</v>
@@ -22616,20 +22616,20 @@
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>126501</v>
+        <v>132801</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Wagga Wagga</t>
+          <t>Warrnambool</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E214" t="n">
         <v>0</v>
@@ -22695,7 +22695,7 @@
         <v>0</v>
       </c>
       <c r="Z214" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA214" t="n">
         <v>0</v>
@@ -22714,29 +22714,29 @@
       </c>
       <c r="AF214" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>126501</v>
+        <v>130291</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Wagga Wagga</t>
+          <t>Werribee</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E215" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F215" t="n">
         <v>0</v>
@@ -22769,7 +22769,7 @@
         <v>0</v>
       </c>
       <c r="P215" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q215" t="n">
         <v>0</v>
@@ -22799,13 +22799,13 @@
         <v>0</v>
       </c>
       <c r="Z215" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA215" t="n">
         <v>0</v>
       </c>
       <c r="AB215" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC215" t="n">
         <v>0</v>
@@ -22818,22 +22818,22 @@
       </c>
       <c r="AF215" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>132801</v>
+        <v>130291</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Warrnambool</t>
+          <t>Werribee</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -22885,7 +22885,7 @@
         <v>0</v>
       </c>
       <c r="T216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U216" t="n">
         <v>0</v>
@@ -22900,10 +22900,10 @@
         <v>0</v>
       </c>
       <c r="Y216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA216" t="n">
         <v>0</v>
@@ -22928,20 +22928,20 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>132801</v>
+        <v>130291</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Warrnambool</t>
+          <t>Werribee</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E217" t="n">
         <v>0</v>
@@ -23004,16 +23004,16 @@
         <v>0</v>
       </c>
       <c r="Y217" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z217" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA217" t="n">
         <v>0</v>
       </c>
       <c r="AB217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC217" t="n">
         <v>0</v>
@@ -23032,20 +23032,20 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>132801</v>
+        <v>130291</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Warrnambool</t>
+          <t>Werribee</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E218" t="n">
         <v>0</v>
@@ -23108,7 +23108,7 @@
         <v>0</v>
       </c>
       <c r="Y218" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Z218" t="n">
         <v>0</v>
@@ -23117,7 +23117,7 @@
         <v>0</v>
       </c>
       <c r="AB218" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC218" t="n">
         <v>0</v>
@@ -23145,83 +23145,83 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>May</t>
         </is>
       </c>
       <c r="D219" t="n">
+        <v>0</v>
+      </c>
+      <c r="E219" t="n">
+        <v>0</v>
+      </c>
+      <c r="F219" t="n">
+        <v>0</v>
+      </c>
+      <c r="G219" t="n">
+        <v>0</v>
+      </c>
+      <c r="H219" t="n">
+        <v>0</v>
+      </c>
+      <c r="I219" t="n">
+        <v>0</v>
+      </c>
+      <c r="J219" t="n">
+        <v>0</v>
+      </c>
+      <c r="K219" t="n">
+        <v>0</v>
+      </c>
+      <c r="L219" t="n">
+        <v>0</v>
+      </c>
+      <c r="M219" t="n">
+        <v>0</v>
+      </c>
+      <c r="N219" t="n">
+        <v>0</v>
+      </c>
+      <c r="O219" t="n">
+        <v>0</v>
+      </c>
+      <c r="P219" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q219" t="n">
+        <v>0</v>
+      </c>
+      <c r="R219" t="n">
+        <v>0</v>
+      </c>
+      <c r="S219" t="n">
+        <v>0</v>
+      </c>
+      <c r="T219" t="n">
+        <v>0</v>
+      </c>
+      <c r="U219" t="n">
+        <v>0</v>
+      </c>
+      <c r="V219" t="n">
+        <v>0</v>
+      </c>
+      <c r="W219" t="n">
+        <v>1</v>
+      </c>
+      <c r="X219" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y219" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z219" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA219" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB219" t="n">
         <v>2</v>
-      </c>
-      <c r="E219" t="n">
-        <v>2</v>
-      </c>
-      <c r="F219" t="n">
-        <v>0</v>
-      </c>
-      <c r="G219" t="n">
-        <v>0</v>
-      </c>
-      <c r="H219" t="n">
-        <v>0</v>
-      </c>
-      <c r="I219" t="n">
-        <v>0</v>
-      </c>
-      <c r="J219" t="n">
-        <v>0</v>
-      </c>
-      <c r="K219" t="n">
-        <v>0</v>
-      </c>
-      <c r="L219" t="n">
-        <v>0</v>
-      </c>
-      <c r="M219" t="n">
-        <v>0</v>
-      </c>
-      <c r="N219" t="n">
-        <v>0</v>
-      </c>
-      <c r="O219" t="n">
-        <v>0</v>
-      </c>
-      <c r="P219" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q219" t="n">
-        <v>0</v>
-      </c>
-      <c r="R219" t="n">
-        <v>0</v>
-      </c>
-      <c r="S219" t="n">
-        <v>0</v>
-      </c>
-      <c r="T219" t="n">
-        <v>0</v>
-      </c>
-      <c r="U219" t="n">
-        <v>0</v>
-      </c>
-      <c r="V219" t="n">
-        <v>0</v>
-      </c>
-      <c r="W219" t="n">
-        <v>0</v>
-      </c>
-      <c r="X219" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y219" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z219" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA219" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB219" t="n">
-        <v>3</v>
       </c>
       <c r="AC219" t="n">
         <v>0</v>
@@ -23249,11 +23249,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E220" t="n">
         <v>0</v>
@@ -23301,7 +23301,7 @@
         <v>0</v>
       </c>
       <c r="T220" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U220" t="n">
         <v>0</v>
@@ -23319,7 +23319,7 @@
         <v>1</v>
       </c>
       <c r="Z220" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA220" t="n">
         <v>0</v>
@@ -23337,422 +23337,6 @@
         <v>0</v>
       </c>
       <c r="AF220" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="n">
-        <v>130291</v>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>Werribee</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="D221" t="n">
-        <v>0</v>
-      </c>
-      <c r="E221" t="n">
-        <v>0</v>
-      </c>
-      <c r="F221" t="n">
-        <v>0</v>
-      </c>
-      <c r="G221" t="n">
-        <v>0</v>
-      </c>
-      <c r="H221" t="n">
-        <v>0</v>
-      </c>
-      <c r="I221" t="n">
-        <v>0</v>
-      </c>
-      <c r="J221" t="n">
-        <v>0</v>
-      </c>
-      <c r="K221" t="n">
-        <v>0</v>
-      </c>
-      <c r="L221" t="n">
-        <v>0</v>
-      </c>
-      <c r="M221" t="n">
-        <v>0</v>
-      </c>
-      <c r="N221" t="n">
-        <v>0</v>
-      </c>
-      <c r="O221" t="n">
-        <v>0</v>
-      </c>
-      <c r="P221" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q221" t="n">
-        <v>0</v>
-      </c>
-      <c r="R221" t="n">
-        <v>0</v>
-      </c>
-      <c r="S221" t="n">
-        <v>0</v>
-      </c>
-      <c r="T221" t="n">
-        <v>0</v>
-      </c>
-      <c r="U221" t="n">
-        <v>0</v>
-      </c>
-      <c r="V221" t="n">
-        <v>0</v>
-      </c>
-      <c r="W221" t="n">
-        <v>0</v>
-      </c>
-      <c r="X221" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y221" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z221" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA221" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB221" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC221" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD221" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE221" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF221" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="n">
-        <v>130291</v>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>Werribee</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>Apr</t>
-        </is>
-      </c>
-      <c r="D222" t="n">
-        <v>0</v>
-      </c>
-      <c r="E222" t="n">
-        <v>0</v>
-      </c>
-      <c r="F222" t="n">
-        <v>0</v>
-      </c>
-      <c r="G222" t="n">
-        <v>0</v>
-      </c>
-      <c r="H222" t="n">
-        <v>0</v>
-      </c>
-      <c r="I222" t="n">
-        <v>0</v>
-      </c>
-      <c r="J222" t="n">
-        <v>0</v>
-      </c>
-      <c r="K222" t="n">
-        <v>0</v>
-      </c>
-      <c r="L222" t="n">
-        <v>0</v>
-      </c>
-      <c r="M222" t="n">
-        <v>0</v>
-      </c>
-      <c r="N222" t="n">
-        <v>0</v>
-      </c>
-      <c r="O222" t="n">
-        <v>0</v>
-      </c>
-      <c r="P222" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q222" t="n">
-        <v>0</v>
-      </c>
-      <c r="R222" t="n">
-        <v>0</v>
-      </c>
-      <c r="S222" t="n">
-        <v>0</v>
-      </c>
-      <c r="T222" t="n">
-        <v>0</v>
-      </c>
-      <c r="U222" t="n">
-        <v>0</v>
-      </c>
-      <c r="V222" t="n">
-        <v>0</v>
-      </c>
-      <c r="W222" t="n">
-        <v>0</v>
-      </c>
-      <c r="X222" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y222" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z222" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA222" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB222" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC222" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD222" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE222" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF222" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="n">
-        <v>130291</v>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>Werribee</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D223" t="n">
-        <v>0</v>
-      </c>
-      <c r="E223" t="n">
-        <v>0</v>
-      </c>
-      <c r="F223" t="n">
-        <v>0</v>
-      </c>
-      <c r="G223" t="n">
-        <v>0</v>
-      </c>
-      <c r="H223" t="n">
-        <v>0</v>
-      </c>
-      <c r="I223" t="n">
-        <v>0</v>
-      </c>
-      <c r="J223" t="n">
-        <v>0</v>
-      </c>
-      <c r="K223" t="n">
-        <v>0</v>
-      </c>
-      <c r="L223" t="n">
-        <v>0</v>
-      </c>
-      <c r="M223" t="n">
-        <v>0</v>
-      </c>
-      <c r="N223" t="n">
-        <v>0</v>
-      </c>
-      <c r="O223" t="n">
-        <v>0</v>
-      </c>
-      <c r="P223" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q223" t="n">
-        <v>0</v>
-      </c>
-      <c r="R223" t="n">
-        <v>0</v>
-      </c>
-      <c r="S223" t="n">
-        <v>0</v>
-      </c>
-      <c r="T223" t="n">
-        <v>0</v>
-      </c>
-      <c r="U223" t="n">
-        <v>0</v>
-      </c>
-      <c r="V223" t="n">
-        <v>0</v>
-      </c>
-      <c r="W223" t="n">
-        <v>1</v>
-      </c>
-      <c r="X223" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y223" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z223" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA223" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB223" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC223" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD223" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE223" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF223" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="n">
-        <v>130291</v>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>Werribee</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>Jun</t>
-        </is>
-      </c>
-      <c r="D224" t="n">
-        <v>0</v>
-      </c>
-      <c r="E224" t="n">
-        <v>0</v>
-      </c>
-      <c r="F224" t="n">
-        <v>0</v>
-      </c>
-      <c r="G224" t="n">
-        <v>0</v>
-      </c>
-      <c r="H224" t="n">
-        <v>0</v>
-      </c>
-      <c r="I224" t="n">
-        <v>0</v>
-      </c>
-      <c r="J224" t="n">
-        <v>0</v>
-      </c>
-      <c r="K224" t="n">
-        <v>0</v>
-      </c>
-      <c r="L224" t="n">
-        <v>0</v>
-      </c>
-      <c r="M224" t="n">
-        <v>0</v>
-      </c>
-      <c r="N224" t="n">
-        <v>0</v>
-      </c>
-      <c r="O224" t="n">
-        <v>0</v>
-      </c>
-      <c r="P224" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q224" t="n">
-        <v>0</v>
-      </c>
-      <c r="R224" t="n">
-        <v>0</v>
-      </c>
-      <c r="S224" t="n">
-        <v>0</v>
-      </c>
-      <c r="T224" t="n">
-        <v>0</v>
-      </c>
-      <c r="U224" t="n">
-        <v>0</v>
-      </c>
-      <c r="V224" t="n">
-        <v>0</v>
-      </c>
-      <c r="W224" t="n">
-        <v>0</v>
-      </c>
-      <c r="X224" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y224" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z224" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA224" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB224" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC224" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD224" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE224" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF224" t="inlineStr">
         <is>
           <t>Active</t>
         </is>

</xml_diff>